<commit_message>
add variable selection lecture to teaching
</commit_message>
<xml_diff>
--- a/cv/cv.xlsx
+++ b/cv/cv.xlsx
@@ -8,18 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cristian/Dropbox/git-repos/cris_blog/cv/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{934D250E-5865-044B-BB01-55671F1B06A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA2868EA-A8D2-3740-8813-5BBF0C03502A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1120" yWindow="680" windowWidth="27660" windowHeight="16460" activeTab="6" xr2:uid="{DA4E0661-7526-1B46-BFDD-FC359AB20183}"/>
+    <workbookView xWindow="1080" yWindow="600" windowWidth="27660" windowHeight="16460" xr2:uid="{DA4E0661-7526-1B46-BFDD-FC359AB20183}"/>
   </bookViews>
   <sheets>
-    <sheet name="employment" sheetId="5" r:id="rId1"/>
-    <sheet name="education" sheetId="1" r:id="rId2"/>
-    <sheet name="research_experience" sheetId="8" r:id="rId3"/>
-    <sheet name="teaching" sheetId="3" r:id="rId4"/>
-    <sheet name="supervision" sheetId="9" r:id="rId5"/>
-    <sheet name="talks" sheetId="6" r:id="rId6"/>
-    <sheet name="grants" sheetId="4" r:id="rId7"/>
+    <sheet name="references" sheetId="10" r:id="rId1"/>
+    <sheet name="organization" sheetId="11" r:id="rId2"/>
+    <sheet name="employment" sheetId="5" r:id="rId3"/>
+    <sheet name="education" sheetId="1" r:id="rId4"/>
+    <sheet name="qualifications" sheetId="8" r:id="rId5"/>
+    <sheet name="teaching" sheetId="3" r:id="rId6"/>
+    <sheet name="supervision" sheetId="9" r:id="rId7"/>
+    <sheet name="talks" sheetId="6" r:id="rId8"/>
+    <sheet name="grants" sheetId="4" r:id="rId9"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -41,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="108">
   <si>
     <t>degree</t>
   </si>
@@ -157,15 +159,9 @@
     <t>position</t>
   </si>
   <si>
-    <t>Inland Norway University of Applied Sciences</t>
-  </si>
-  <si>
     <t>Norway</t>
   </si>
   <si>
-    <t>Norwegian School of Sports Science</t>
-  </si>
-  <si>
     <t>The Netherlands</t>
   </si>
   <si>
@@ -193,18 +189,6 @@
     <t>Danish Reproducibility Network meetup</t>
   </si>
   <si>
-    <t>Research internship (unpaid)</t>
-  </si>
-  <si>
-    <t>2015-2016</t>
-  </si>
-  <si>
-    <t>Universiry of Granada</t>
-  </si>
-  <si>
-    <t>Spain</t>
-  </si>
-  <si>
     <t>China</t>
   </si>
   <si>
@@ -217,15 +201,6 @@
     <t>Technological University of Dublin</t>
   </si>
   <si>
-    <t>Co-supervised four students creating a tool to extract sample sizes from published studies</t>
-  </si>
-  <si>
-    <t>Taught R Markdown for reproducible reporting and data simulation for statistical analysis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Taught anatomy </t>
-  </si>
-  <si>
     <t>2021-2025</t>
   </si>
   <si>
@@ -253,22 +228,7 @@
     <t>2024-Present</t>
   </si>
   <si>
-    <t>Lecturer of Behaveoral Research Methods 3</t>
-  </si>
-  <si>
-    <t>Teaching assistant of Behaveoral Research Methods 3</t>
-  </si>
-  <si>
     <t>Supervisor of Master End Project</t>
-  </si>
-  <si>
-    <t>Co-supervised a meta-analysis project examining the impact of school sanitation on students' academic performance</t>
-  </si>
-  <si>
-    <t>Co-supervised a project using automated search extraction to extract and attempted hypotheses using large language models</t>
-  </si>
-  <si>
-    <t>Co-supervised the development of a tool to identify incorrect use of the standard error of measurement instead of the standard deviation in effect size calculations for meta-analyses</t>
   </si>
   <si>
     <t>Workshop on Metacheck</t>
@@ -324,21 +284,6 @@
     <t xml:space="preserve"> Taught multiple regression and power analysis.</t>
   </si>
   <si>
-    <t>Taught introduction to meta-analysis</t>
-  </si>
-  <si>
-    <t>Assisted students during tutorial sessions with course assignments</t>
-  </si>
-  <si>
-    <t>Investigated the effects of two HIIT protocols on VO₂max in highly trained cyclists using physiological assessments, including lactate threshold, VO₂max, and cycling economy testing.</t>
-  </si>
-  <si>
-    <t>Contributed to race analysis and the assessment of swimmers' dry-land performance profiles and propulsive force.</t>
-  </si>
-  <si>
-    <t>Investigated the use of the 1080 Sprint resistance device in swimming to measure power–velocity profiles and estimate drag characteristics in swimmers.</t>
-  </si>
-  <si>
     <t>Funding to develop an R package designed to assist master's students and supervisors in performing automatic checks to enforce best research practices.</t>
   </si>
   <si>
@@ -376,6 +321,75 @@
   </si>
   <si>
     <t>My PhD thesis examined the factors hindering replicability and reproducibility  in sports and exercise science.</t>
+  </si>
+  <si>
+    <t>Lecturer of Advanced Research Methods and Research Ethics</t>
+  </si>
+  <si>
+    <t>Teaching assistant of Advanced Research Methods and Research Ethics</t>
+  </si>
+  <si>
+    <t>Start to Supervise</t>
+  </si>
+  <si>
+    <t>Co-supervised a project creating an automated tool that categorizs repository files based on the file name, index detected variables and their labels, and reconstruct the repository into an established standard.</t>
+  </si>
+  <si>
+    <t>Co-supervised a project using automated search extraction to extract and attempted hypotheses using large language models.</t>
+  </si>
+  <si>
+    <t>Co-supervised a meta-analysis project examining the impact of school sanitation on students' academic performance.</t>
+  </si>
+  <si>
+    <t>Co-supervised the development of a tool to identify incorrect use of the standard error of measurement instead of the standard deviation in effect size calculations for meta-analyses.</t>
+  </si>
+  <si>
+    <t>Taught introduction to meta-analysis.</t>
+  </si>
+  <si>
+    <t>Assisted students during tutorial sessions with course assignments.</t>
+  </si>
+  <si>
+    <t>Taught R Markdown for reproducible reporting and data simulation for statistical analysis.</t>
+  </si>
+  <si>
+    <t>Taught anatomy.</t>
+  </si>
+  <si>
+    <t>Enabling Course for main supervisors.</t>
+  </si>
+  <si>
+    <t>reference</t>
+  </si>
+  <si>
+    <t>Collaborator</t>
+  </si>
+  <si>
+    <t>Technological University Dublin</t>
+  </si>
+  <si>
+    <t>Dublin, Ireland</t>
+  </si>
+  <si>
+    <t>Galway, Ireland</t>
+  </si>
+  <si>
+    <t>Atlantic Technological University Galway</t>
+  </si>
+  <si>
+    <t>Transparency, Technology and AI in peer review Conference</t>
+  </si>
+  <si>
+    <t>I co-organized a one-day conference that brought together different stakeholders to discuss the role of transparency, technology, and AI in peer review (https://meta-eindhoven.github.io/events/).</t>
+  </si>
+  <si>
+    <t>Joe Warne (joe.warne@tudublin.ie)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PhD supervisor </t>
+  </si>
+  <si>
+    <t>Jennifer Muprhy (jennifer.murphy@atu.ie)</t>
   </si>
 </sst>
 </file>
@@ -439,7 +453,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -475,13 +489,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -797,6 +814,112 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F2265E7-B48C-CF42-951E-B253301EB0D2}">
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="47" customHeight="1" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="4" width="37.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="14" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="47" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="47" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>101</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A70E321-D466-8649-BB94-B1AFF1BE8269}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="27.6640625" style="7" customWidth="1"/>
+    <col min="2" max="2" width="16.1640625" style="7" customWidth="1"/>
+    <col min="3" max="3" width="35" style="7" customWidth="1"/>
+    <col min="4" max="4" width="33.33203125" style="7" customWidth="1"/>
+    <col min="5" max="5" width="64.5" style="7" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="66" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="B2" s="3">
+        <v>2026</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="16" t="s">
+        <v>104</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA4DFF70-337C-994E-B0CC-B59ADAD82018}">
   <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -839,7 +962,7 @@
         <v>7</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>102</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" ht="34" x14ac:dyDescent="0.2">
@@ -847,7 +970,7 @@
         <v>8</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>6</v>
@@ -856,7 +979,7 @@
         <v>7</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>103</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -864,7 +987,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66DB8938-134D-9E48-B807-361AEFF395A1}">
   <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -898,7 +1021,7 @@
         <v>21</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>6</v>
@@ -907,7 +1030,7 @@
         <v>7</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>100</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" ht="34" x14ac:dyDescent="0.2">
@@ -924,7 +1047,7 @@
         <v>10</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>99</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" ht="34" x14ac:dyDescent="0.2">
@@ -941,7 +1064,7 @@
         <v>17</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>98</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" ht="34" x14ac:dyDescent="0.2">
@@ -958,7 +1081,7 @@
         <v>13</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>101</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -966,14 +1089,15 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17D0B757-8294-AE49-A8E3-ACF99479B5EF}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26.1640625" customWidth="1"/>
     <col min="3" max="3" width="39" customWidth="1"/>
-    <col min="5" max="5" width="81.6640625" style="15" customWidth="1"/>
+    <col min="4" max="4" width="16.1640625" customWidth="1"/>
+    <col min="5" max="5" width="81.6640625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -989,59 +1113,25 @@
       <c r="D1" t="s">
         <v>27</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="10" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="10" t="s">
-        <v>50</v>
+        <v>87</v>
       </c>
       <c r="B2" s="10">
-        <v>2018</v>
+        <v>2026</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>40</v>
+        <v>6</v>
       </c>
       <c r="D2" s="10" t="s">
         <v>39</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" s="10" customFormat="1" ht="43" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="B3" s="10">
-        <v>2017</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" s="10" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A4" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="E4" s="13" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -1049,7 +1139,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{531F101D-2B48-9F46-A53F-FA67ACC31D52}">
   <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1079,70 +1169,70 @@
     </row>
     <row r="2" spans="1:5" s="6" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>5</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>84</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="6" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>5</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="6" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="6" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>71</v>
+        <v>86</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D5" s="3">
         <v>2024</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="6" customFormat="1" ht="34" x14ac:dyDescent="0.2">
@@ -1153,21 +1243,21 @@
         <v>6</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D6" s="3">
         <v>2024</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>59</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="6" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A7" s="8" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>36</v>
@@ -1176,7 +1266,7 @@
         <v>2021</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>60</v>
+        <v>95</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.2">
@@ -1191,7 +1281,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A0F6311-6111-6149-8D98-BE8A9A017CC2}">
   <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1220,72 +1310,72 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="6" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" s="6" customFormat="1" ht="85" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D2" s="3">
-        <v>2025</v>
+        <v>39</v>
+      </c>
+      <c r="D2" s="7">
+        <v>2026</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="6" customFormat="1" ht="51" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>25</v>
+        <v>61</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D3" s="3">
         <v>2025</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" s="6" customFormat="1" ht="68" x14ac:dyDescent="0.2">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" s="6" customFormat="1" ht="51" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>72</v>
+        <v>25</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D4" s="3">
+        <v>2025</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" s="6" customFormat="1" ht="68" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D5" s="3">
         <v>2024</v>
       </c>
-      <c r="E4" s="5" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" s="6" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D5" s="3">
-        <v>2023</v>
-      </c>
       <c r="E5" s="5" t="s">
-        <v>58</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -1293,7 +1383,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A465BE91-A970-8F4B-854C-C3F13E65FCA4}">
   <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1302,7 +1392,7 @@
     <col min="2" max="2" width="17.83203125" style="4" customWidth="1"/>
     <col min="3" max="3" width="24.5" style="4" customWidth="1"/>
     <col min="4" max="4" width="16.1640625" style="4" customWidth="1"/>
-    <col min="5" max="5" width="47.5" style="14" customWidth="1"/>
+    <col min="5" max="5" width="47.5" style="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1318,30 +1408,30 @@
       <c r="D1" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="E1" s="14" t="s">
+      <c r="E1" s="13" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="B2" s="4">
         <v>2026</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>93</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="B3" s="4">
         <v>2026</v>
@@ -1353,63 +1443,63 @@
         <v>32</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>94</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="12" customFormat="1" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="B4" s="5">
         <v>2025</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>95</v>
+        <v>53</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" ht="51" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="B5" s="5">
         <v>2025</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="E5" s="14" t="s">
-        <v>96</v>
+        <v>42</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="2" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B6" s="5">
         <v>2025</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="E6" s="14" t="s">
-        <v>97</v>
+        <v>44</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="2" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B7" s="5">
         <v>2025</v>
@@ -1420,8 +1510,8 @@
       <c r="D7" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="14" t="s">
-        <v>97</v>
+      <c r="E7" s="13" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="2" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.2">
@@ -1437,8 +1527,8 @@
       <c r="D8" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="E8" s="14" t="s">
-        <v>80</v>
+      <c r="E8" s="13" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="2" customFormat="1" ht="51" x14ac:dyDescent="0.2">
@@ -1455,12 +1545,12 @@
         <v>32</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="2" customFormat="1" ht="51" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>34</v>
@@ -1472,24 +1562,24 @@
         <v>36</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>81</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B11" s="5">
         <v>2019</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
     </row>
     <row r="18" spans="3:3" x14ac:dyDescent="0.2">
@@ -1500,7 +1590,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47C77CB8-88D5-B640-9A7F-46D72B331807}">
   <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1527,16 +1617,16 @@
     </row>
     <row r="2" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="B2" s="3">
         <v>2026</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>92</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:4" s="2" customFormat="1" ht="51" x14ac:dyDescent="0.2">
@@ -1550,7 +1640,7 @@
         <v>6</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>